<commit_message>
Planilla de jornaleros, hoja Reporte: sin las columnas CONTROL TRELLO y la del legajo repetido. El control del Resumen «Registros sin OK en Trello» (leía esa columna) se saca de la plantilla; la tabla de controles queda en 4 filas.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/jornaleros.xlsx
+++ b/server/plantillas/jornaleros.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">LIQUIDACION!$A$3:$J$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Reporte!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SUBTOTAL!$A$1:$L$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Resumen Ejecutivo'!$B$2:$N$76</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Resumen Ejecutivo'!$B$2:$N$75</definedName>
   </definedNames>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
@@ -2609,7 +2609,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:S76"/>
+  <dimension ref="A2:S75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2" style="30" customWidth="1"/>
@@ -3906,13 +3906,13 @@
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.3">
       <c r="C73" s="45" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D73" s="65">
-        <f>COUNT(Reporte!$K$2:$K$1000)-COUNTIFS(Reporte!$M$2:$M$1000,"OK",Reporte!$K$2:$K$1000,"&lt;&gt;")</f>
+        <f>ROUND(IFERROR(INDEX(LIQUIDACION!$E:$E,IFERROR(MATCH("Total general",LIQUIDACION!$B:$B,0),MATCH("Total Result",LIQUIDACION!$B:$B,0))),0)-F7,0)</f>
       </c>
       <c r="E73" s="92">
-        <f>IF(D73=0,"✓ OK","⚠ Hay registros sin validar en Trello")</f>
+        <f>IF(D73=0,"✓ Tabla dinámica actualizada","⚠ Actualizar la tabla dinámica de LIQUIDACION")</f>
       </c>
       <c r="F73" s="105"/>
       <c r="G73" s="105"/>
@@ -3924,49 +3924,29 @@
       <c r="M73" s="105"/>
       <c r="N73" s="105"/>
     </row>
-    <row r="74" spans="2:19" x14ac:dyDescent="0.3">
-      <c r="C74" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="D74" s="65">
-        <f>ROUND(IFERROR(INDEX(LIQUIDACION!$E:$E,IFERROR(MATCH("Total general",LIQUIDACION!$B:$B,0),MATCH("Total Result",LIQUIDACION!$B:$B,0))),0)-F7,0)</f>
-      </c>
-      <c r="E74" s="92">
-        <f>IF(D74=0,"✓ Tabla dinámica actualizada","⚠ Actualizar la tabla dinámica de LIQUIDACION")</f>
-      </c>
-      <c r="F74" s="105"/>
-      <c r="G74" s="105"/>
-      <c r="H74" s="105"/>
-      <c r="I74" s="105"/>
-      <c r="J74" s="105"/>
-      <c r="K74" s="105"/>
-      <c r="L74" s="105"/>
-      <c r="M74" s="105"/>
-      <c r="N74" s="105"/>
-    </row>
-    <row r="76" spans="2:19" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="110" t="s">
+    <row r="75" spans="2:19" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B75" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="C76" s="98"/>
-      <c r="D76" s="98"/>
-      <c r="E76" s="98"/>
-      <c r="F76" s="98"/>
-      <c r="G76" s="98"/>
-      <c r="H76" s="98"/>
-      <c r="I76" s="98"/>
-      <c r="J76" s="98"/>
-      <c r="K76" s="98"/>
-      <c r="L76" s="98"/>
-      <c r="M76" s="98"/>
-      <c r="N76" s="98"/>
+      <c r="C75" s="98"/>
+      <c r="D75" s="98"/>
+      <c r="E75" s="98"/>
+      <c r="F75" s="98"/>
+      <c r="G75" s="98"/>
+      <c r="H75" s="98"/>
+      <c r="I75" s="98"/>
+      <c r="J75" s="98"/>
+      <c r="K75" s="98"/>
+      <c r="L75" s="98"/>
+      <c r="M75" s="98"/>
+      <c r="N75" s="98"/>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="49">
     <mergeCell ref="E70:N70"/>
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="J63:N64"/>
-    <mergeCell ref="B76:N76"/>
+    <mergeCell ref="B75:N75"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="J53:N53"/>
     <mergeCell ref="M54:N54"/>
@@ -3975,7 +3955,6 @@
     <mergeCell ref="J56:L56"/>
     <mergeCell ref="L6:N6"/>
     <mergeCell ref="E73:N73"/>
-    <mergeCell ref="E74:N74"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="J55:L55"/>
     <mergeCell ref="B68:N68"/>
@@ -4014,7 +3993,7 @@
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="F10:G10"/>
   </mergeCells>
-  <conditionalFormatting sqref="E70:E74">
+  <conditionalFormatting sqref="E70:E73">
     <cfRule type="expression" dxfId="27" priority="1">
       <formula>LEFT($E70,1)="✓"</formula>
     </cfRule>
@@ -4049,11 +4028,9 @@
     <col min="10" max="10" width="16.5" style="30" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.3984375" style="30" customWidth="1"/>
     <col min="12" max="12" width="12.09765625" style="30" customWidth="1"/>
-    <col min="13" max="13" width="17.796875" style="30" customWidth="1"/>
-    <col min="14" max="14" width="33.296875" style="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
@@ -4089,9 +4066,6 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>